<commit_message>
Merge origin/main into main
Conflicts:
	src/java/vbsp/ims/khnv2021/excel/ExcelExport.java
</commit_message>
<xml_diff>
--- a/web/EXCEL_TEMPLATE/KHNV/KHNV_DK01A.xlsx
+++ b/web/EXCEL_TEMPLATE/KHNV/KHNV_DK01A.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\GIT\IMS_REPORTS\build\web\EXCEL_TEMPLATE\KHNV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09EAEAC2-96F6-4ADA-BE0B-F4698C0FA684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7FE30E-B530-4D3A-890C-693F0DB5BC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11280" xr2:uid="{FEA2E927-87FC-4F8F-B922-B59702A7794E}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="DK_01A" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">DK_01A!$A$1:$G$101</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">DK_01A!$A$1:$G$171</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">DK_01A!$8:$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -381,14 +381,26 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -409,18 +421,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -740,7 +740,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J187"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="1" customWidth="1"/>
@@ -1069,127 +1069,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F1" s="20" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="20"/>
+      <c r="F1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="21"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
-      <c r="F2" s="30" t="s">
+      <c r="F2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="30"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="3"/>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
     </row>
     <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
     </row>
     <row r="6" spans="1:10" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="23" t="s">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="26" t="s">
+      <c r="F9" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="27"/>
+      <c r="G9" s="31"/>
     </row>
     <row r="10" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="21"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="28" t="s">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="32" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="21"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
     </row>
     <row r="12" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="5">
@@ -1233,12 +1233,12 @@
       <c r="C14" s="14"/>
       <c r="D14" s="16"/>
       <c r="E14" s="17">
-        <f t="shared" ref="E14:E77" si="0">D14+F14</f>
+        <f t="shared" ref="E14:E134" si="0">D14+F14</f>
         <v>0</v>
       </c>
       <c r="F14" s="18"/>
       <c r="G14" s="17">
-        <f t="shared" ref="G14:G77" si="1">IFERROR(F14/D14*100,0)</f>
+        <f t="shared" ref="G14:G134" si="1">IFERROR(F14/D14*100,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -1617,11 +1617,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="15"/>
       <c r="B40" s="15"/>
       <c r="C40" s="14"/>
-      <c r="D40" s="16"/>
+      <c r="D40" s="18"/>
       <c r="E40" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1632,11 +1632,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="15"/>
       <c r="B41" s="15"/>
       <c r="C41" s="14"/>
-      <c r="D41" s="16"/>
+      <c r="D41" s="18"/>
       <c r="E41" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1647,11 +1647,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="15"/>
       <c r="B42" s="15"/>
       <c r="C42" s="14"/>
-      <c r="D42" s="16"/>
+      <c r="D42" s="18"/>
       <c r="E42" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1662,11 +1662,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A43" s="15"/>
       <c r="B43" s="15"/>
       <c r="C43" s="14"/>
-      <c r="D43" s="16"/>
+      <c r="D43" s="18"/>
       <c r="E43" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1677,11 +1677,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A44" s="15"/>
       <c r="B44" s="15"/>
       <c r="C44" s="14"/>
-      <c r="D44" s="16"/>
+      <c r="D44" s="18"/>
       <c r="E44" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1692,11 +1692,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A45" s="15"/>
       <c r="B45" s="15"/>
       <c r="C45" s="14"/>
-      <c r="D45" s="16"/>
+      <c r="D45" s="18"/>
       <c r="E45" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1707,11 +1707,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
       <c r="C46" s="14"/>
-      <c r="D46" s="16"/>
+      <c r="D46" s="18"/>
       <c r="E46" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1722,11 +1722,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
       <c r="C47" s="14"/>
-      <c r="D47" s="16"/>
+      <c r="D47" s="18"/>
       <c r="E47" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1737,11 +1737,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
       <c r="C48" s="14"/>
-      <c r="D48" s="16"/>
+      <c r="D48" s="18"/>
       <c r="E48" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1752,11 +1752,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A49" s="15"/>
       <c r="B49" s="15"/>
       <c r="C49" s="14"/>
-      <c r="D49" s="16"/>
+      <c r="D49" s="18"/>
       <c r="E49" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1767,11 +1767,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A50" s="15"/>
       <c r="B50" s="15"/>
       <c r="C50" s="14"/>
-      <c r="D50" s="16"/>
+      <c r="D50" s="18"/>
       <c r="E50" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1782,11 +1782,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="15"/>
       <c r="C51" s="14"/>
-      <c r="D51" s="16"/>
+      <c r="D51" s="18"/>
       <c r="E51" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1797,11 +1797,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="15"/>
       <c r="C52" s="14"/>
-      <c r="D52" s="16"/>
+      <c r="D52" s="18"/>
       <c r="E52" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1812,11 +1812,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A53" s="15"/>
       <c r="B53" s="15"/>
       <c r="C53" s="14"/>
-      <c r="D53" s="16"/>
+      <c r="D53" s="18"/>
       <c r="E53" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1827,11 +1827,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A54" s="15"/>
       <c r="B54" s="15"/>
       <c r="C54" s="14"/>
-      <c r="D54" s="16"/>
+      <c r="D54" s="18"/>
       <c r="E54" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1842,11 +1842,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A55" s="15"/>
       <c r="B55" s="15"/>
       <c r="C55" s="14"/>
-      <c r="D55" s="16"/>
+      <c r="D55" s="18"/>
       <c r="E55" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1857,11 +1857,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A56" s="15"/>
       <c r="B56" s="15"/>
       <c r="C56" s="14"/>
-      <c r="D56" s="16"/>
+      <c r="D56" s="18"/>
       <c r="E56" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1872,11 +1872,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A57" s="15"/>
       <c r="B57" s="15"/>
       <c r="C57" s="14"/>
-      <c r="D57" s="16"/>
+      <c r="D57" s="18"/>
       <c r="E57" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1887,11 +1887,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A58" s="15"/>
       <c r="B58" s="15"/>
       <c r="C58" s="14"/>
-      <c r="D58" s="16"/>
+      <c r="D58" s="18"/>
       <c r="E58" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1902,11 +1902,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A59" s="15"/>
       <c r="B59" s="15"/>
       <c r="C59" s="14"/>
-      <c r="D59" s="16"/>
+      <c r="D59" s="18"/>
       <c r="E59" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1917,11 +1917,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A60" s="15"/>
       <c r="B60" s="15"/>
       <c r="C60" s="14"/>
-      <c r="D60" s="16"/>
+      <c r="D60" s="18"/>
       <c r="E60" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1932,11 +1932,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A61" s="15"/>
       <c r="B61" s="15"/>
       <c r="C61" s="14"/>
-      <c r="D61" s="16"/>
+      <c r="D61" s="18"/>
       <c r="E61" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1947,11 +1947,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A62" s="15"/>
       <c r="B62" s="15"/>
       <c r="C62" s="14"/>
-      <c r="D62" s="16"/>
+      <c r="D62" s="18"/>
       <c r="E62" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1962,11 +1962,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A63" s="15"/>
       <c r="B63" s="15"/>
       <c r="C63" s="14"/>
-      <c r="D63" s="16"/>
+      <c r="D63" s="18"/>
       <c r="E63" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1977,11 +1977,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A64" s="15"/>
       <c r="B64" s="15"/>
       <c r="C64" s="14"/>
-      <c r="D64" s="16"/>
+      <c r="D64" s="18"/>
       <c r="E64" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1992,11 +1992,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A65" s="15"/>
       <c r="B65" s="15"/>
       <c r="C65" s="14"/>
-      <c r="D65" s="16"/>
+      <c r="D65" s="18"/>
       <c r="E65" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2007,11 +2007,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A66" s="15"/>
       <c r="B66" s="15"/>
       <c r="C66" s="14"/>
-      <c r="D66" s="16"/>
+      <c r="D66" s="18"/>
       <c r="E66" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2022,11 +2022,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A67" s="15"/>
       <c r="B67" s="15"/>
       <c r="C67" s="14"/>
-      <c r="D67" s="16"/>
+      <c r="D67" s="18"/>
       <c r="E67" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2037,11 +2037,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A68" s="15"/>
       <c r="B68" s="15"/>
       <c r="C68" s="14"/>
-      <c r="D68" s="16"/>
+      <c r="D68" s="18"/>
       <c r="E68" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2052,11 +2052,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A69" s="15"/>
       <c r="B69" s="15"/>
       <c r="C69" s="14"/>
-      <c r="D69" s="16"/>
+      <c r="D69" s="18"/>
       <c r="E69" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2067,11 +2067,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A70" s="15"/>
       <c r="B70" s="15"/>
       <c r="C70" s="14"/>
-      <c r="D70" s="16"/>
+      <c r="D70" s="18"/>
       <c r="E70" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2082,11 +2082,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A71" s="15"/>
       <c r="B71" s="15"/>
       <c r="C71" s="14"/>
-      <c r="D71" s="16"/>
+      <c r="D71" s="18"/>
       <c r="E71" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2097,11 +2097,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A72" s="15"/>
       <c r="B72" s="15"/>
       <c r="C72" s="14"/>
-      <c r="D72" s="16"/>
+      <c r="D72" s="18"/>
       <c r="E72" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2112,11 +2112,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A73" s="15"/>
       <c r="B73" s="15"/>
       <c r="C73" s="14"/>
-      <c r="D73" s="16"/>
+      <c r="D73" s="18"/>
       <c r="E73" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2127,11 +2127,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A74" s="15"/>
       <c r="B74" s="15"/>
       <c r="C74" s="14"/>
-      <c r="D74" s="16"/>
+      <c r="D74" s="18"/>
       <c r="E74" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2142,11 +2142,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A75" s="15"/>
       <c r="B75" s="15"/>
       <c r="C75" s="14"/>
-      <c r="D75" s="16"/>
+      <c r="D75" s="18"/>
       <c r="E75" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2157,11 +2157,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A76" s="15"/>
       <c r="B76" s="15"/>
       <c r="C76" s="14"/>
-      <c r="D76" s="16"/>
+      <c r="D76" s="18"/>
       <c r="E76" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2172,11 +2172,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A77" s="15"/>
       <c r="B77" s="15"/>
       <c r="C77" s="14"/>
-      <c r="D77" s="16"/>
+      <c r="D77" s="18"/>
       <c r="E77" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2187,108 +2187,108 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A78" s="15"/>
       <c r="B78" s="15"/>
       <c r="C78" s="14"/>
-      <c r="D78" s="16"/>
+      <c r="D78" s="18"/>
       <c r="E78" s="17">
-        <f t="shared" ref="E78:E96" si="2">D78+F78</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F78" s="18"/>
       <c r="G78" s="17">
-        <f t="shared" ref="G78:G96" si="3">IFERROR(F78/D78*100,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A79" s="15"/>
       <c r="B79" s="15"/>
       <c r="C79" s="14"/>
-      <c r="D79" s="16"/>
+      <c r="D79" s="18"/>
       <c r="E79" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F79" s="18"/>
       <c r="G79" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A80" s="15"/>
       <c r="B80" s="15"/>
       <c r="C80" s="14"/>
-      <c r="D80" s="16"/>
+      <c r="D80" s="18"/>
       <c r="E80" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F80" s="18"/>
       <c r="G80" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A81" s="15"/>
       <c r="B81" s="15"/>
       <c r="C81" s="14"/>
-      <c r="D81" s="16"/>
+      <c r="D81" s="18"/>
       <c r="E81" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F81" s="18"/>
       <c r="G81" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A82" s="15"/>
       <c r="B82" s="15"/>
       <c r="C82" s="14"/>
-      <c r="D82" s="16"/>
+      <c r="D82" s="18"/>
       <c r="E82" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F82" s="18"/>
       <c r="G82" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A83" s="15"/>
       <c r="B83" s="15"/>
       <c r="C83" s="14"/>
-      <c r="D83" s="16"/>
+      <c r="D83" s="18"/>
       <c r="E83" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F83" s="18"/>
       <c r="G83" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A84" s="15"/>
       <c r="B84" s="15"/>
       <c r="C84" s="14"/>
-      <c r="D84" s="16"/>
+      <c r="D84" s="18"/>
       <c r="E84" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F84" s="18"/>
       <c r="G84" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2296,14 +2296,14 @@
       <c r="A85" s="15"/>
       <c r="B85" s="15"/>
       <c r="C85" s="14"/>
-      <c r="D85" s="16"/>
+      <c r="D85" s="18"/>
       <c r="E85" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F85" s="18"/>
       <c r="G85" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2311,14 +2311,14 @@
       <c r="A86" s="15"/>
       <c r="B86" s="15"/>
       <c r="C86" s="14"/>
-      <c r="D86" s="16"/>
+      <c r="D86" s="18"/>
       <c r="E86" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F86" s="18"/>
       <c r="G86" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2326,14 +2326,14 @@
       <c r="A87" s="15"/>
       <c r="B87" s="15"/>
       <c r="C87" s="14"/>
-      <c r="D87" s="16"/>
+      <c r="D87" s="18"/>
       <c r="E87" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F87" s="18"/>
       <c r="G87" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2341,14 +2341,14 @@
       <c r="A88" s="15"/>
       <c r="B88" s="15"/>
       <c r="C88" s="14"/>
-      <c r="D88" s="16"/>
+      <c r="D88" s="18"/>
       <c r="E88" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F88" s="18"/>
       <c r="G88" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2356,14 +2356,14 @@
       <c r="A89" s="15"/>
       <c r="B89" s="15"/>
       <c r="C89" s="14"/>
-      <c r="D89" s="16"/>
+      <c r="D89" s="18"/>
       <c r="E89" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F89" s="18"/>
       <c r="G89" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2371,14 +2371,14 @@
       <c r="A90" s="15"/>
       <c r="B90" s="15"/>
       <c r="C90" s="14"/>
-      <c r="D90" s="16"/>
+      <c r="D90" s="18"/>
       <c r="E90" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F90" s="18"/>
       <c r="G90" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2386,14 +2386,14 @@
       <c r="A91" s="15"/>
       <c r="B91" s="15"/>
       <c r="C91" s="14"/>
-      <c r="D91" s="16"/>
+      <c r="D91" s="18"/>
       <c r="E91" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F91" s="18"/>
       <c r="G91" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2401,14 +2401,14 @@
       <c r="A92" s="15"/>
       <c r="B92" s="15"/>
       <c r="C92" s="14"/>
-      <c r="D92" s="16"/>
+      <c r="D92" s="18"/>
       <c r="E92" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F92" s="18"/>
       <c r="G92" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2416,14 +2416,14 @@
       <c r="A93" s="15"/>
       <c r="B93" s="15"/>
       <c r="C93" s="14"/>
-      <c r="D93" s="16"/>
+      <c r="D93" s="18"/>
       <c r="E93" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F93" s="18"/>
       <c r="G93" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2431,14 +2431,14 @@
       <c r="A94" s="15"/>
       <c r="B94" s="15"/>
       <c r="C94" s="14"/>
-      <c r="D94" s="16"/>
+      <c r="D94" s="18"/>
       <c r="E94" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F94" s="18"/>
       <c r="G94" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2446,14 +2446,14 @@
       <c r="A95" s="15"/>
       <c r="B95" s="15"/>
       <c r="C95" s="14"/>
-      <c r="D95" s="16"/>
+      <c r="D95" s="18"/>
       <c r="E95" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F95" s="18"/>
       <c r="G95" s="17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -2461,128 +2461,1171 @@
       <c r="A96" s="15"/>
       <c r="B96" s="15"/>
       <c r="C96" s="14"/>
-      <c r="D96" s="16"/>
+      <c r="D96" s="18"/>
       <c r="E96" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F96" s="18"/>
       <c r="G96" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A97" s="15"/>
+      <c r="B97" s="15"/>
+      <c r="C97" s="14"/>
+      <c r="D97" s="16"/>
+      <c r="E97" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F97" s="18"/>
+      <c r="G97" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A98" s="15"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="14"/>
+      <c r="D98" s="16"/>
+      <c r="E98" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F98" s="18"/>
+      <c r="G98" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A99" s="15"/>
+      <c r="B99" s="15"/>
+      <c r="C99" s="14"/>
+      <c r="D99" s="16"/>
+      <c r="E99" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F99" s="18"/>
+      <c r="G99" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A100" s="15"/>
+      <c r="B100" s="15"/>
+      <c r="C100" s="14"/>
+      <c r="D100" s="16"/>
+      <c r="E100" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F100" s="18"/>
+      <c r="G100" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A101" s="15"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="14"/>
+      <c r="D101" s="16"/>
+      <c r="E101" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F101" s="18"/>
+      <c r="G101" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A102" s="15"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="14"/>
+      <c r="D102" s="16"/>
+      <c r="E102" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F102" s="18"/>
+      <c r="G102" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A103" s="15"/>
+      <c r="B103" s="15"/>
+      <c r="C103" s="14"/>
+      <c r="D103" s="16"/>
+      <c r="E103" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F103" s="18"/>
+      <c r="G103" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A104" s="15"/>
+      <c r="B104" s="15"/>
+      <c r="C104" s="14"/>
+      <c r="D104" s="16"/>
+      <c r="E104" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F104" s="18"/>
+      <c r="G104" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A105" s="15"/>
+      <c r="B105" s="15"/>
+      <c r="C105" s="14"/>
+      <c r="D105" s="16"/>
+      <c r="E105" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F105" s="18"/>
+      <c r="G105" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A106" s="15"/>
+      <c r="B106" s="15"/>
+      <c r="C106" s="14"/>
+      <c r="D106" s="16"/>
+      <c r="E106" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F106" s="18"/>
+      <c r="G106" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A107" s="15"/>
+      <c r="B107" s="15"/>
+      <c r="C107" s="14"/>
+      <c r="D107" s="16"/>
+      <c r="E107" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F107" s="18"/>
+      <c r="G107" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A108" s="15"/>
+      <c r="B108" s="15"/>
+      <c r="C108" s="14"/>
+      <c r="D108" s="16"/>
+      <c r="E108" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F108" s="18"/>
+      <c r="G108" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A109" s="15"/>
+      <c r="B109" s="15"/>
+      <c r="C109" s="14"/>
+      <c r="D109" s="16"/>
+      <c r="E109" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F109" s="18"/>
+      <c r="G109" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A110" s="15"/>
+      <c r="B110" s="15"/>
+      <c r="C110" s="14"/>
+      <c r="D110" s="16"/>
+      <c r="E110" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F110" s="18"/>
+      <c r="G110" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A111" s="15"/>
+      <c r="B111" s="15"/>
+      <c r="C111" s="14"/>
+      <c r="D111" s="16"/>
+      <c r="E111" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F111" s="18"/>
+      <c r="G111" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A112" s="15"/>
+      <c r="B112" s="15"/>
+      <c r="C112" s="14"/>
+      <c r="D112" s="16"/>
+      <c r="E112" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F112" s="18"/>
+      <c r="G112" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A113" s="15"/>
+      <c r="B113" s="15"/>
+      <c r="C113" s="14"/>
+      <c r="D113" s="16"/>
+      <c r="E113" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F113" s="18"/>
+      <c r="G113" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A114" s="15"/>
+      <c r="B114" s="15"/>
+      <c r="C114" s="14"/>
+      <c r="D114" s="16"/>
+      <c r="E114" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F114" s="18"/>
+      <c r="G114" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A115" s="15"/>
+      <c r="B115" s="15"/>
+      <c r="C115" s="14"/>
+      <c r="D115" s="16"/>
+      <c r="E115" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F115" s="18"/>
+      <c r="G115" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A116" s="15"/>
+      <c r="B116" s="15"/>
+      <c r="C116" s="14"/>
+      <c r="D116" s="16"/>
+      <c r="E116" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F116" s="18"/>
+      <c r="G116" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A117" s="15"/>
+      <c r="B117" s="15"/>
+      <c r="C117" s="14"/>
+      <c r="D117" s="16"/>
+      <c r="E117" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F117" s="18"/>
+      <c r="G117" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A118" s="15"/>
+      <c r="B118" s="15"/>
+      <c r="C118" s="14"/>
+      <c r="D118" s="16"/>
+      <c r="E118" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F118" s="18"/>
+      <c r="G118" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A119" s="15"/>
+      <c r="B119" s="15"/>
+      <c r="C119" s="14"/>
+      <c r="D119" s="16"/>
+      <c r="E119" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F119" s="18"/>
+      <c r="G119" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A120" s="15"/>
+      <c r="B120" s="15"/>
+      <c r="C120" s="14"/>
+      <c r="D120" s="16"/>
+      <c r="E120" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F120" s="18"/>
+      <c r="G120" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A121" s="15"/>
+      <c r="B121" s="15"/>
+      <c r="C121" s="14"/>
+      <c r="D121" s="16"/>
+      <c r="E121" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F121" s="18"/>
+      <c r="G121" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A122" s="15"/>
+      <c r="B122" s="15"/>
+      <c r="C122" s="14"/>
+      <c r="D122" s="16"/>
+      <c r="E122" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F122" s="18"/>
+      <c r="G122" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A123" s="15"/>
+      <c r="B123" s="15"/>
+      <c r="C123" s="14"/>
+      <c r="D123" s="16"/>
+      <c r="E123" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F123" s="18"/>
+      <c r="G123" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A124" s="15"/>
+      <c r="B124" s="15"/>
+      <c r="C124" s="14"/>
+      <c r="D124" s="16"/>
+      <c r="E124" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F124" s="18"/>
+      <c r="G124" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A125" s="15"/>
+      <c r="B125" s="15"/>
+      <c r="C125" s="14"/>
+      <c r="D125" s="16"/>
+      <c r="E125" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F125" s="18"/>
+      <c r="G125" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A126" s="15"/>
+      <c r="B126" s="15"/>
+      <c r="C126" s="14"/>
+      <c r="D126" s="16"/>
+      <c r="E126" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F126" s="18"/>
+      <c r="G126" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A127" s="15"/>
+      <c r="B127" s="15"/>
+      <c r="C127" s="14"/>
+      <c r="D127" s="16"/>
+      <c r="E127" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F127" s="18"/>
+      <c r="G127" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A128" s="15"/>
+      <c r="B128" s="15"/>
+      <c r="C128" s="14"/>
+      <c r="D128" s="16"/>
+      <c r="E128" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F128" s="18"/>
+      <c r="G128" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A129" s="15"/>
+      <c r="B129" s="15"/>
+      <c r="C129" s="14"/>
+      <c r="D129" s="16"/>
+      <c r="E129" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F129" s="18"/>
+      <c r="G129" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A130" s="15"/>
+      <c r="B130" s="15"/>
+      <c r="C130" s="14"/>
+      <c r="D130" s="16"/>
+      <c r="E130" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F130" s="18"/>
+      <c r="G130" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A131" s="15"/>
+      <c r="B131" s="15"/>
+      <c r="C131" s="14"/>
+      <c r="D131" s="16"/>
+      <c r="E131" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F131" s="18"/>
+      <c r="G131" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A132" s="15"/>
+      <c r="B132" s="15"/>
+      <c r="C132" s="14"/>
+      <c r="D132" s="16"/>
+      <c r="E132" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F132" s="18"/>
+      <c r="G132" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A133" s="15"/>
+      <c r="B133" s="15"/>
+      <c r="C133" s="14"/>
+      <c r="D133" s="16"/>
+      <c r="E133" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F133" s="18"/>
+      <c r="G133" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A134" s="15"/>
+      <c r="B134" s="15"/>
+      <c r="C134" s="14"/>
+      <c r="D134" s="16"/>
+      <c r="E134" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F134" s="18"/>
+      <c r="G134" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A135" s="15"/>
+      <c r="B135" s="15"/>
+      <c r="C135" s="14"/>
+      <c r="D135" s="16"/>
+      <c r="E135" s="17">
+        <f t="shared" ref="E135:E166" si="2">D135+F135</f>
+        <v>0</v>
+      </c>
+      <c r="F135" s="18"/>
+      <c r="G135" s="17">
+        <f t="shared" ref="G135:G166" si="3">IFERROR(F135/D135*100,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A136" s="15"/>
+      <c r="B136" s="15"/>
+      <c r="C136" s="14"/>
+      <c r="D136" s="16"/>
+      <c r="E136" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F136" s="18"/>
+      <c r="G136" s="17">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A97" s="8"/>
-      <c r="B97" s="8"/>
-      <c r="C97" s="9"/>
-      <c r="G97" s="6"/>
-    </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A98" s="8"/>
-      <c r="B98" s="8"/>
-      <c r="C98" s="1" t="s">
+    <row r="137" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A137" s="15"/>
+      <c r="B137" s="15"/>
+      <c r="C137" s="14"/>
+      <c r="D137" s="16"/>
+      <c r="E137" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F137" s="18"/>
+      <c r="G137" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A138" s="15"/>
+      <c r="B138" s="15"/>
+      <c r="C138" s="14"/>
+      <c r="D138" s="16"/>
+      <c r="E138" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F138" s="18"/>
+      <c r="G138" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A139" s="15"/>
+      <c r="B139" s="15"/>
+      <c r="C139" s="14"/>
+      <c r="D139" s="16"/>
+      <c r="E139" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F139" s="18"/>
+      <c r="G139" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A140" s="15"/>
+      <c r="B140" s="15"/>
+      <c r="C140" s="14"/>
+      <c r="D140" s="16"/>
+      <c r="E140" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F140" s="18"/>
+      <c r="G140" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A141" s="15"/>
+      <c r="B141" s="15"/>
+      <c r="C141" s="14"/>
+      <c r="D141" s="18"/>
+      <c r="E141" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F141" s="18"/>
+      <c r="G141" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A142" s="15"/>
+      <c r="B142" s="15"/>
+      <c r="C142" s="14"/>
+      <c r="D142" s="18"/>
+      <c r="E142" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F142" s="18"/>
+      <c r="G142" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A143" s="15"/>
+      <c r="B143" s="15"/>
+      <c r="C143" s="14"/>
+      <c r="D143" s="18"/>
+      <c r="E143" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F143" s="18"/>
+      <c r="G143" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A144" s="15"/>
+      <c r="B144" s="15"/>
+      <c r="C144" s="14"/>
+      <c r="D144" s="18"/>
+      <c r="E144" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F144" s="18"/>
+      <c r="G144" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A145" s="15"/>
+      <c r="B145" s="15"/>
+      <c r="C145" s="14"/>
+      <c r="D145" s="18"/>
+      <c r="E145" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F145" s="18"/>
+      <c r="G145" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A146" s="15"/>
+      <c r="B146" s="15"/>
+      <c r="C146" s="14"/>
+      <c r="D146" s="18"/>
+      <c r="E146" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F146" s="18"/>
+      <c r="G146" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A147" s="15"/>
+      <c r="B147" s="15"/>
+      <c r="C147" s="14"/>
+      <c r="D147" s="18"/>
+      <c r="E147" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F147" s="18"/>
+      <c r="G147" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A148" s="15"/>
+      <c r="B148" s="15"/>
+      <c r="C148" s="14"/>
+      <c r="D148" s="18"/>
+      <c r="E148" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F148" s="18"/>
+      <c r="G148" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A149" s="15"/>
+      <c r="B149" s="15"/>
+      <c r="C149" s="14"/>
+      <c r="D149" s="18"/>
+      <c r="E149" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F149" s="18"/>
+      <c r="G149" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A150" s="15"/>
+      <c r="B150" s="15"/>
+      <c r="C150" s="14"/>
+      <c r="D150" s="18"/>
+      <c r="E150" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F150" s="18"/>
+      <c r="G150" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A151" s="15"/>
+      <c r="B151" s="15"/>
+      <c r="C151" s="14"/>
+      <c r="D151" s="18"/>
+      <c r="E151" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F151" s="18"/>
+      <c r="G151" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A152" s="15"/>
+      <c r="B152" s="15"/>
+      <c r="C152" s="14"/>
+      <c r="D152" s="18"/>
+      <c r="E152" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F152" s="18"/>
+      <c r="G152" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A153" s="15"/>
+      <c r="B153" s="15"/>
+      <c r="C153" s="14"/>
+      <c r="D153" s="18"/>
+      <c r="E153" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F153" s="18"/>
+      <c r="G153" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" s="6" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A154" s="15"/>
+      <c r="B154" s="15"/>
+      <c r="C154" s="14"/>
+      <c r="D154" s="16"/>
+      <c r="E154" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F154" s="18"/>
+      <c r="G154" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A155" s="15"/>
+      <c r="B155" s="15"/>
+      <c r="C155" s="14"/>
+      <c r="D155" s="16"/>
+      <c r="E155" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F155" s="18"/>
+      <c r="G155" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A156" s="15"/>
+      <c r="B156" s="15"/>
+      <c r="C156" s="14"/>
+      <c r="D156" s="16"/>
+      <c r="E156" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F156" s="18"/>
+      <c r="G156" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A157" s="15"/>
+      <c r="B157" s="15"/>
+      <c r="C157" s="14"/>
+      <c r="D157" s="16"/>
+      <c r="E157" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F157" s="18"/>
+      <c r="G157" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A158" s="15"/>
+      <c r="B158" s="15"/>
+      <c r="C158" s="14"/>
+      <c r="D158" s="16"/>
+      <c r="E158" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F158" s="18"/>
+      <c r="G158" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A159" s="15"/>
+      <c r="B159" s="15"/>
+      <c r="C159" s="14"/>
+      <c r="D159" s="16"/>
+      <c r="E159" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F159" s="18"/>
+      <c r="G159" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A160" s="15"/>
+      <c r="B160" s="15"/>
+      <c r="C160" s="14"/>
+      <c r="D160" s="16"/>
+      <c r="E160" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F160" s="18"/>
+      <c r="G160" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A161" s="15"/>
+      <c r="B161" s="15"/>
+      <c r="C161" s="14"/>
+      <c r="D161" s="16"/>
+      <c r="E161" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F161" s="18"/>
+      <c r="G161" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A162" s="15"/>
+      <c r="B162" s="15"/>
+      <c r="C162" s="14"/>
+      <c r="D162" s="16"/>
+      <c r="E162" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F162" s="18"/>
+      <c r="G162" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A163" s="15"/>
+      <c r="B163" s="15"/>
+      <c r="C163" s="14"/>
+      <c r="D163" s="16"/>
+      <c r="E163" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F163" s="18"/>
+      <c r="G163" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A164" s="15"/>
+      <c r="B164" s="15"/>
+      <c r="C164" s="14"/>
+      <c r="D164" s="16"/>
+      <c r="E164" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F164" s="18"/>
+      <c r="G164" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A165" s="15"/>
+      <c r="B165" s="15"/>
+      <c r="C165" s="14"/>
+      <c r="D165" s="16"/>
+      <c r="E165" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F165" s="18"/>
+      <c r="G165" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A166" s="15"/>
+      <c r="B166" s="15"/>
+      <c r="C166" s="14"/>
+      <c r="D166" s="16"/>
+      <c r="E166" s="17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F166" s="18"/>
+      <c r="G166" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A167" s="8"/>
+      <c r="B167" s="8"/>
+      <c r="C167" s="9"/>
+      <c r="G167" s="6"/>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A168" s="8"/>
+      <c r="B168" s="8"/>
+      <c r="C168" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G98" s="6"/>
-    </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A99" s="10"/>
-      <c r="B99" s="10"/>
-      <c r="C99" s="10"/>
-      <c r="D99" s="19" t="s">
+      <c r="G168" s="6"/>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A169" s="10"/>
+      <c r="B169" s="10"/>
+      <c r="C169" s="10"/>
+      <c r="D169" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E99" s="19"/>
-      <c r="F99" s="19"/>
-      <c r="G99" s="19"/>
-    </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A100" s="11"/>
-      <c r="B100" s="11"/>
-      <c r="C100" s="12" t="s">
+      <c r="E169" s="25"/>
+      <c r="F169" s="25"/>
+      <c r="G169" s="25"/>
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A170" s="11"/>
+      <c r="B170" s="11"/>
+      <c r="C170" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D100" s="20"/>
-      <c r="E100" s="20"/>
-      <c r="F100" s="20"/>
-      <c r="G100" s="20"/>
-      <c r="H100" s="11"/>
-      <c r="I100" s="11"/>
-      <c r="J100" s="11"/>
-    </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A101" s="9"/>
-      <c r="B101" s="9"/>
-      <c r="C101" s="8" t="s">
+      <c r="D170" s="21"/>
+      <c r="E170" s="21"/>
+      <c r="F170" s="21"/>
+      <c r="G170" s="21"/>
+      <c r="H170" s="11"/>
+      <c r="I170" s="11"/>
+      <c r="J170" s="11"/>
+    </row>
+    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A171" s="9"/>
+      <c r="B171" s="9"/>
+      <c r="C171" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D101" s="19"/>
-      <c r="E101" s="19"/>
-      <c r="F101" s="19"/>
-      <c r="G101" s="19"/>
-      <c r="H101" s="13"/>
-      <c r="I101" s="13"/>
-      <c r="J101" s="13"/>
-    </row>
-    <row r="102" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A102" s="2"/>
-      <c r="B102" s="2"/>
-      <c r="C102" s="2"/>
-      <c r="D102" s="2"/>
-      <c r="E102" s="2"/>
-      <c r="F102" s="2"/>
-    </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C107" s="11" t="s">
+      <c r="D171" s="25"/>
+      <c r="E171" s="25"/>
+      <c r="F171" s="25"/>
+      <c r="G171" s="25"/>
+      <c r="H171" s="13"/>
+      <c r="I171" s="13"/>
+      <c r="J171" s="13"/>
+    </row>
+    <row r="172" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A172" s="2"/>
+      <c r="B172" s="2"/>
+      <c r="C172" s="2"/>
+      <c r="D172" s="2"/>
+      <c r="E172" s="2"/>
+      <c r="F172" s="2"/>
+    </row>
+    <row r="177" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C177" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C108" s="1" t="s">
+    <row r="178" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C178" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C109" s="1" t="s">
+    <row r="179" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C179" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C110" s="1" t="s">
+    <row r="180" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C180" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C111" s="1" t="s">
+    <row r="181" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C181" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C112" s="1" t="s">
+    <row r="182" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C182" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="114" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C114" s="1" t="s">
+    <row r="184" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C184" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="117" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C117" s="11"/>
+    <row r="187" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C187" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="B8:B11"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="D3:G3"/>
-    <mergeCell ref="D4:G4"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="D99:G99"/>
-    <mergeCell ref="D100:G100"/>
-    <mergeCell ref="D101:G101"/>
+    <mergeCell ref="D169:G169"/>
+    <mergeCell ref="D170:G170"/>
+    <mergeCell ref="D171:G171"/>
     <mergeCell ref="E7:H7"/>
     <mergeCell ref="A8:A11"/>
     <mergeCell ref="C8:C11"/>
@@ -2592,6 +3635,13 @@
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="G10:G11"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="D3:G3"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.19685039370078741" bottom="3.937007874015748E-2" header="3.937007874015748E-2" footer="3.937007874015748E-2"/>

</xml_diff>